<commit_message>
Docs for MVP version 2
</commit_message>
<xml_diff>
--- a/Docs/MVP/MVP_Development_Backlog.xlsx
+++ b/Docs/MVP/MVP_Development_Backlog.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="1" r:id="R19af60339a7449aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="1" r:id="Rfc51f28c956848e5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -129,7 +129,7 @@
         <x:color rgb="FF256029"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9EAD3"/>
         </x:patternFill>
       </x:fill>
@@ -140,7 +140,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
@@ -151,7 +151,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -162,7 +162,7 @@
         <x:color rgb="FF1F4E78"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9EAF7"/>
         </x:patternFill>
       </x:fill>
@@ -173,7 +173,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE1E1"/>
         </x:patternFill>
       </x:fill>
@@ -184,7 +184,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF1CC"/>
         </x:patternFill>
       </x:fill>
@@ -412,8 +412,8 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="25" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="42" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="10" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="11" hidden="0" customWidth="1"/>
@@ -426,7 +426,7 @@
   <x:sheetData>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="2" t="str">
-        <x:v>SER594 Dungeon MVP Development Backlog</x:v>
+        <x:v>SER594 Dungeon Vertical Slice v2.0 Development Backlog</x:v>
       </x:c>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
@@ -483,7 +483,7 @@
     <x:row r="4" ht="24" customHeight="1"/>
     <x:row r="5" ht="24" customHeight="1">
       <x:c r="A5" s="7" t="str">
-        <x:v>Planning basis: MVP Game Design and Requirements Specification v1.0. Owners and schedules are team inputs.</x:v>
+        <x:v>Planning basis: MVP Vertical Slice Game Design and Requirements Specification v2.0. D&amp;D combat and follow-up skills are retained ideas, not MVP tasks.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
@@ -540,16 +540,16 @@
       <x:c r="F8" s="16" t="str">
         <x:v>S</x:v>
       </x:c>
-      <x:c r="G8" s="14" t="str"/>
+      <x:c r="G8" s="14"/>
       <x:c r="H8" s="14" t="str">
         <x:v>Tech Lead</x:v>
       </x:c>
-      <x:c r="I8" s="15" t="str"/>
+      <x:c r="I8" s="15"/>
       <x:c r="J8" s="17" t="str">
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="K8" s="14" t="str">
-        <x:v>The policy is documented and all team members use the same project setting.</x:v>
+        <x:v>The policy is documented and every team member uses the same project setting.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
@@ -577,12 +577,12 @@
       <x:c r="H9" s="14" t="str">
         <x:v>Tech Lead</x:v>
       </x:c>
-      <x:c r="I9" s="15" t="str"/>
+      <x:c r="I9" s="15"/>
       <x:c r="J9" s="17" t="str">
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="K9" s="14" t="str">
-        <x:v>The agreed folders exist and the current SampleScene still opens without missing references.</x:v>
+        <x:v>The agreed folders exist and SampleScene still opens without missing references.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
@@ -596,7 +596,7 @@
         <x:v>Scenes</x:v>
       </x:c>
       <x:c r="D10" s="14" t="str">
-        <x:v>Create Bootstrap, MainMenu, RouteMap, Combat, and RunComplete scenes.</x:v>
+        <x:v>Create Bootstrap, MainMenu, DungeonRoom, and RunComplete scenes.</x:v>
       </x:c>
       <x:c r="E10" s="16" t="str">
         <x:v>P0</x:v>
@@ -610,7 +610,7 @@
       <x:c r="H10" s="14" t="str">
         <x:v>Unity Generalist</x:v>
       </x:c>
-      <x:c r="I10" s="15" t="str"/>
+      <x:c r="I10" s="15"/>
       <x:c r="J10" s="17" t="str">
         <x:v>Not Started</x:v>
       </x:c>
@@ -629,13 +629,13 @@
         <x:v>Core State</x:v>
       </x:c>
       <x:c r="D11" s="14" t="str">
-        <x:v>Implement GameSession and the mutable RunState and PlayerRunState models.</x:v>
+        <x:v>Implement GameSession plus RunState, PartyState, CharacterRunState, and RoomRuntimeState.</x:v>
       </x:c>
       <x:c r="E11" s="16" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F11" s="16" t="str">
-        <x:v>M</x:v>
+        <x:v>L</x:v>
       </x:c>
       <x:c r="G11" s="14" t="str">
         <x:v>SET-02</x:v>
@@ -643,12 +643,12 @@
       <x:c r="H11" s="14" t="str">
         <x:v>Systems</x:v>
       </x:c>
-      <x:c r="I11" s="15" t="str"/>
+      <x:c r="I11" s="15"/>
       <x:c r="J11" s="17" t="str">
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="K11" s="14" t="str">
-        <x:v>One authoritative run state survives scene changes and initializes with the approved values.</x:v>
+        <x:v>One authoritative run state survives scene changes and supports four party records.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="42" customHeight="1">
@@ -662,7 +662,7 @@
         <x:v>Scene Flow</x:v>
       </x:c>
       <x:c r="D12" s="14" t="str">
-        <x:v>Implement valid scene transitions through a SceneFlowService.</x:v>
+        <x:v>Implement valid menu, room, door, completion, and reset transitions through SceneFlowService.</x:v>
       </x:c>
       <x:c r="E12" s="16" t="str">
         <x:v>P0</x:v>
@@ -676,12 +676,12 @@
       <x:c r="H12" s="14" t="str">
         <x:v>Systems</x:v>
       </x:c>
-      <x:c r="I12" s="15" t="str"/>
+      <x:c r="I12" s="15"/>
       <x:c r="J12" s="17" t="str">
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="K12" s="14" t="str">
-        <x:v>The application can move from Bootstrap to MainMenu and start a clean run without duplicate services.</x:v>
+        <x:v>The application transitions without duplicate services and starts a clean run after reset.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
@@ -695,13 +695,13 @@
         <x:v>Data</x:v>
       </x:c>
       <x:c r="D13" s="14" t="str">
-        <x:v>Define player, enemy, boss, potion, and weapon data structures.</x:v>
+        <x:v>Define ScriptableObject types for rooms, characters, equipment, skills, enemies, events, Inherent Skills, rewards, and optional environment interactions.</x:v>
       </x:c>
       <x:c r="E13" s="16" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F13" s="16" t="str">
-        <x:v>M</x:v>
+        <x:v>L</x:v>
       </x:c>
       <x:c r="G13" s="14" t="str">
         <x:v>SET-04</x:v>
@@ -714,87 +714,87 @@
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="K13" s="14" t="str">
-        <x:v>All approved MVP values are represented once and can be read by runtime systems.</x:v>
+        <x:v>Each static concept has one editable definition and mutable state is stored separately.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
       <x:c r="A14" s="13" t="str">
-        <x:v>DATA-02</x:v>
+        <x:v>ROOM-01</x:v>
       </x:c>
       <x:c r="B14" s="13" t="str">
-        <x:v>M0 Foundation</x:v>
+        <x:v>M1 Rooms and Exploration</x:v>
       </x:c>
       <x:c r="C14" s="13" t="str">
-        <x:v>Data</x:v>
+        <x:v>Room Model</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
-        <x:v>Create static definitions or configuration assets for enemies, items, events, and combat.</x:v>
+        <x:v>Implement RoomDefinition, module sockets, door sockets, battle anchors, and optional interaction sockets.</x:v>
       </x:c>
       <x:c r="E14" s="16" t="str">
-        <x:v>P1</x:v>
+        <x:v>P0</x:v>
       </x:c>
       <x:c r="F14" s="16" t="str">
-        <x:v>M</x:v>
+        <x:v>L</x:v>
       </x:c>
       <x:c r="G14" s="14" t="str">
         <x:v>DATA-01</x:v>
       </x:c>
       <x:c r="H14" s="14" t="str">
-        <x:v>Systems</x:v>
+        <x:v>Room Systems</x:v>
       </x:c>
       <x:c r="I14" s="15" t="str"/>
       <x:c r="J14" s="17" t="str">
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="K14" s="14" t="str">
-        <x:v>Design values can be edited without changing unrelated runtime logic.</x:v>
+        <x:v>A room definition identifies every required socket and can leave optional interaction sockets unused.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="42" customHeight="1">
       <x:c r="A15" s="13" t="str">
-        <x:v>FLOW-01</x:v>
+        <x:v>ROOM-02</x:v>
       </x:c>
       <x:c r="B15" s="13" t="str">
-        <x:v>M1 Game Flow</x:v>
+        <x:v>M1 Rooms and Exploration</x:v>
       </x:c>
       <x:c r="C15" s="13" t="str">
-        <x:v>Stage Flow</x:v>
+        <x:v>Room Assembly</x:v>
       </x:c>
       <x:c r="D15" s="14" t="str">
-        <x:v>Implement StageGenerator for Stage 1-1, Stages 1-2 to 1-4, and Stage 1-5.</x:v>
+        <x:v>Build the reusable DungeonRoom scene and assemble authored modules from a RoomDefinition.</x:v>
       </x:c>
       <x:c r="E15" s="16" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F15" s="16" t="str">
-        <x:v>M</x:v>
+        <x:v>L</x:v>
       </x:c>
       <x:c r="G15" s="14" t="str">
-        <x:v>SET-04</x:v>
+        <x:v>SET-03, ROOM-01</x:v>
       </x:c>
       <x:c r="H15" s="14" t="str">
-        <x:v>Systems</x:v>
-      </x:c>
-      <x:c r="I15" s="15" t="str"/>
+        <x:v>Room Systems</x:v>
+      </x:c>
+      <x:c r="I15" s="15"/>
       <x:c r="J15" s="17" t="str">
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="K15" s="14" t="str">
-        <x:v>Generated choices follow fixed-stage, exclusion, distinct-choice, and combat-repeat rules.</x:v>
+        <x:v>One scene loads a valid room with required and optional modules at authored sockets.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="42" customHeight="1">
       <x:c r="A16" s="13" t="str">
-        <x:v>FLOW-02</x:v>
+        <x:v>ROOM-03</x:v>
       </x:c>
       <x:c r="B16" s="13" t="str">
-        <x:v>M1 Game Flow</x:v>
+        <x:v>M1 Rooms and Exploration</x:v>
       </x:c>
       <x:c r="C16" s="13" t="str">
-        <x:v>Route UI</x:v>
+        <x:v>Doors</x:v>
       </x:c>
       <x:c r="D16" s="14" t="str">
-        <x:v>Build the route-selection screen and connect node buttons to the active run.</x:v>
+        <x:v>Implement physical door interaction, connection data, and current-room progression.</x:v>
       </x:c>
       <x:c r="E16" s="16" t="str">
         <x:v>P0</x:v>
@@ -803,229 +803,229 @@
         <x:v>M</x:v>
       </x:c>
       <x:c r="G16" s="14" t="str">
-        <x:v>FLOW-01, SET-05</x:v>
+        <x:v>ROOM-02, SET-05</x:v>
       </x:c>
       <x:c r="H16" s="14" t="str">
-        <x:v>UI</x:v>
-      </x:c>
-      <x:c r="I16" s="15" t="str"/>
+        <x:v>Room Systems</x:v>
+      </x:c>
+      <x:c r="I16" s="15"/>
       <x:c r="J16" s="17" t="str">
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="K16" s="14" t="str">
-        <x:v>The screen displays the correct number and type of choices and records one legal selection.</x:v>
+        <x:v>Using an available door records the room state and loads exactly one connected room.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="42" customHeight="1">
       <x:c r="A17" s="13" t="str">
-        <x:v>FLOW-03</x:v>
+        <x:v>ROOM-04</x:v>
       </x:c>
       <x:c r="B17" s="13" t="str">
-        <x:v>M1 Game Flow</x:v>
+        <x:v>M1 Rooms and Exploration</x:v>
       </x:c>
       <x:c r="C17" s="13" t="str">
-        <x:v>Run Lifecycle</x:v>
+        <x:v>Exploration</x:v>
       </x:c>
       <x:c r="D17" s="14" t="str">
-        <x:v>Implement new-run initialization, run abandonment, and return-to-menu reset.</x:v>
+        <x:v>Adapt or replace prototype movement with Input System leader exploration and camera bounds.</x:v>
       </x:c>
       <x:c r="E17" s="16" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F17" s="16" t="str">
-        <x:v>M</x:v>
+        <x:v>L</x:v>
       </x:c>
       <x:c r="G17" s="14" t="str">
-        <x:v>SET-04, SET-05</x:v>
+        <x:v>SET-01, ROOM-02</x:v>
       </x:c>
       <x:c r="H17" s="14" t="str">
-        <x:v>Systems</x:v>
-      </x:c>
-      <x:c r="I17" s="15" t="str"/>
+        <x:v>Exploration</x:v>
+      </x:c>
+      <x:c r="I17" s="15"/>
       <x:c r="J17" s="17" t="str">
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="K17" s="14" t="str">
-        <x:v>Starting or abandoning a run produces a clean state with no values from the prior run.</x:v>
+        <x:v>The selected leader can explore one room reliably with no legacy-input dependency in new code.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="42" customHeight="1">
       <x:c r="A18" s="13" t="str">
-        <x:v>HEX-01</x:v>
+        <x:v>ROOM-05</x:v>
       </x:c>
       <x:c r="B18" s="13" t="str">
-        <x:v>M2 Hex Grid</x:v>
+        <x:v>M1 Rooms and Exploration</x:v>
       </x:c>
       <x:c r="C18" s="13" t="str">
-        <x:v>Hex Math</x:v>
+        <x:v>Interaction</x:v>
       </x:c>
       <x:c r="D18" s="14" t="str">
-        <x:v>Implement axial hex coordinates, equality, neighbors, and distance.</x:v>
+        <x:v>Implement focus detection, prompts, and typed interaction commands for doors, NPCs, chests, events, and approved optional interactions.</x:v>
       </x:c>
       <x:c r="E18" s="16" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F18" s="16" t="str">
-        <x:v>M</x:v>
+        <x:v>L</x:v>
       </x:c>
       <x:c r="G18" s="14" t="str">
-        <x:v>SET-02</x:v>
+        <x:v>ROOM-02, ROOM-04</x:v>
       </x:c>
       <x:c r="H18" s="14" t="str">
-        <x:v>Combat Systems</x:v>
+        <x:v>Exploration</x:v>
       </x:c>
       <x:c r="I18" s="15" t="str"/>
       <x:c r="J18" s="17" t="str">
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="K18" s="14" t="str">
-        <x:v>Hex coordinate operations return correct deterministic results in EditMode tests.</x:v>
+        <x:v>Only the focused valid target accepts one interaction and gives readable feedback.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="42" customHeight="1">
       <x:c r="A19" s="13" t="str">
-        <x:v>HEX-02</x:v>
+        <x:v>ROOM-06</x:v>
       </x:c>
       <x:c r="B19" s="13" t="str">
-        <x:v>M2 Hex Grid</x:v>
+        <x:v>M1 Rooms and Exploration</x:v>
       </x:c>
       <x:c r="C19" s="13" t="str">
-        <x:v>Board Generation</x:v>
+        <x:v>Party Presentation</x:v>
       </x:c>
       <x:c r="D19" s="14" t="str">
-        <x:v>Generate the pointy-topped radius-3 combat board.</x:v>
+        <x:v>Display only the selected leader during exploration and support changing the leader outside combat.</x:v>
       </x:c>
       <x:c r="E19" s="16" t="str">
-        <x:v>P0</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="F19" s="16" t="str">
         <x:v>M</x:v>
       </x:c>
       <x:c r="G19" s="14" t="str">
-        <x:v>HEX-01</x:v>
+        <x:v>SET-04, ROOM-04</x:v>
       </x:c>
       <x:c r="H19" s="14" t="str">
-        <x:v>Combat Systems</x:v>
-      </x:c>
-      <x:c r="I19" s="15" t="str"/>
+        <x:v>Exploration</x:v>
+      </x:c>
+      <x:c r="I19" s="15"/>
       <x:c r="J19" s="17" t="str">
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="K19" s="14" t="str">
-        <x:v>The generated board contains exactly 37 unique hexes.</x:v>
+        <x:v>Changing the leader swaps the exploration model while the full party remains in runtime state and HUD.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="42" customHeight="1">
       <x:c r="A20" s="13" t="str">
-        <x:v>HEX-03</x:v>
+        <x:v>ROOM-07</x:v>
       </x:c>
       <x:c r="B20" s="13" t="str">
-        <x:v>M2 Hex Grid</x:v>
+        <x:v>M1 Rooms and Exploration</x:v>
       </x:c>
       <x:c r="C20" s="13" t="str">
-        <x:v>Board Presentation</x:v>
+        <x:v>Vertical Slice Rooms</x:v>
       </x:c>
       <x:c r="D20" s="14" t="str">
-        <x:v>Convert axial coordinates to world positions and render selectable hex visuals.</x:v>
+        <x:v>Author three connected rooms with mixed modules and a final boss room.</x:v>
       </x:c>
       <x:c r="E20" s="16" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F20" s="16" t="str">
-        <x:v>M</x:v>
+        <x:v>L</x:v>
       </x:c>
       <x:c r="G20" s="14" t="str">
-        <x:v>HEX-02</x:v>
+        <x:v>ROOM-02, ROOM-03, ROOM-05</x:v>
       </x:c>
       <x:c r="H20" s="14" t="str">
-        <x:v>Combat Systems</x:v>
-      </x:c>
-      <x:c r="I20" s="15" t="str"/>
+        <x:v>Level Design</x:v>
+      </x:c>
+      <x:c r="I20" s="15"/>
       <x:c r="J20" s="17" t="str">
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="K20" s="14" t="str">
-        <x:v>Every logical hex has one correctly positioned visual and click target.</x:v>
+        <x:v>The run contains three playable rooms, two to three doors where applicable, and mixed content.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="42" customHeight="1">
       <x:c r="A21" s="13" t="str">
-        <x:v>HEX-04</x:v>
+        <x:v>PARTY-01</x:v>
       </x:c>
       <x:c r="B21" s="13" t="str">
-        <x:v>M2 Hex Grid</x:v>
+        <x:v>M2 Party and Loadouts</x:v>
       </x:c>
       <x:c r="C21" s="13" t="str">
-        <x:v>Movement</x:v>
+        <x:v>Party</x:v>
       </x:c>
       <x:c r="D21" s="14" t="str">
-        <x:v>Calculate reachable cells and display legal movement highlights.</x:v>
+        <x:v>Initialize two playable party members while keeping capacity for four.</x:v>
       </x:c>
       <x:c r="E21" s="16" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F21" s="16" t="str">
-        <x:v>L</x:v>
+        <x:v>M</x:v>
       </x:c>
       <x:c r="G21" s="14" t="str">
-        <x:v>HEX-01, HEX-03</x:v>
+        <x:v>SET-04, DATA-01</x:v>
       </x:c>
       <x:c r="H21" s="14" t="str">
-        <x:v>Combat Systems</x:v>
-      </x:c>
-      <x:c r="I21" s="15" t="str"/>
+        <x:v>Systems</x:v>
+      </x:c>
+      <x:c r="I21" s="15"/>
       <x:c r="J21" s="17" t="str">
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="K21" s="14" t="str">
-        <x:v>A unit with movement 3 sees only legal unoccupied destinations within range.</x:v>
+        <x:v>A new run creates two active members and the data model accepts up to four without redesign.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="42" customHeight="1">
       <x:c r="A22" s="13" t="str">
-        <x:v>HEX-05</x:v>
+        <x:v>PARTY-02</x:v>
       </x:c>
       <x:c r="B22" s="13" t="str">
-        <x:v>M2 Hex Grid</x:v>
+        <x:v>M2 Party and Loadouts</x:v>
       </x:c>
       <x:c r="C22" s="13" t="str">
-        <x:v>Pathfinding</x:v>
+        <x:v>Character Identity</x:v>
       </x:c>
       <x:c r="D22" s="14" t="str">
-        <x:v>Implement occupancy checks and shortest-path movement for the enemy.</x:v>
+        <x:v>Define base stats, proficiency tendencies, growth caps, and identity passive data for each playable character.</x:v>
       </x:c>
       <x:c r="E22" s="16" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F22" s="16" t="str">
-        <x:v>L</x:v>
+        <x:v>M</x:v>
       </x:c>
       <x:c r="G22" s="14" t="str">
-        <x:v>HEX-04</x:v>
+        <x:v>PARTY-01</x:v>
       </x:c>
       <x:c r="H22" s="14" t="str">
-        <x:v>Combat Systems</x:v>
-      </x:c>
-      <x:c r="I22" s="15" t="str"/>
+        <x:v>Design and Systems</x:v>
+      </x:c>
+      <x:c r="I22" s="15"/>
       <x:c r="J22" s="17" t="str">
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="K22" s="14" t="str">
-        <x:v>The enemy reaches the closest legal hex without entering occupied or invalid cells.</x:v>
+        <x:v>The two characters remain mechanically different after exchanging configurable equipment.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="42" customHeight="1">
       <x:c r="A23" s="13" t="str">
-        <x:v>COM-01</x:v>
+        <x:v>LOAD-01</x:v>
       </x:c>
       <x:c r="B23" s="13" t="str">
-        <x:v>M3 Combat</x:v>
+        <x:v>M2 Party and Loadouts</x:v>
       </x:c>
       <x:c r="C23" s="13" t="str">
-        <x:v>Combat Flow</x:v>
+        <x:v>Weapons</x:v>
       </x:c>
       <x:c r="D23" s="14" t="str">
-        <x:v>Implement CombatController and explicit combat phases.</x:v>
+        <x:v>Implement Active and Secondary weapon slots, weapon tags, and one free switch at turn start.</x:v>
       </x:c>
       <x:c r="E23" s="16" t="str">
         <x:v>P0</x:v>
@@ -1034,163 +1034,163 @@
         <x:v>L</x:v>
       </x:c>
       <x:c r="G23" s="14" t="str">
-        <x:v>SET-04, HEX-02</x:v>
+        <x:v>PARTY-01, DATA-01</x:v>
       </x:c>
       <x:c r="H23" s="14" t="str">
         <x:v>Combat Systems</x:v>
       </x:c>
-      <x:c r="I23" s="15" t="str"/>
+      <x:c r="I23" s="15"/>
       <x:c r="J23" s="17" t="str">
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="K23" s="14" t="str">
-        <x:v>Only valid phase transitions occur and one controller owns the active turn.</x:v>
+        <x:v>Each character equips two weapons and changes the active weapon only at the allowed timing.</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="42" customHeight="1">
       <x:c r="A24" s="13" t="str">
-        <x:v>COM-02</x:v>
+        <x:v>SKILL-01</x:v>
       </x:c>
       <x:c r="B24" s="13" t="str">
-        <x:v>M3 Combat</x:v>
+        <x:v>M2 Party and Loadouts</x:v>
       </x:c>
       <x:c r="C24" s="13" t="str">
-        <x:v>Initiative</x:v>
+        <x:v>Active Skills</x:v>
       </x:c>
       <x:c r="D24" s="14" t="str">
-        <x:v>Implement D20 initiative with rerolls on ties.</x:v>
+        <x:v>Implement selectable active-skill loadouts and equipped-weapon tag requirements.</x:v>
       </x:c>
       <x:c r="E24" s="16" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F24" s="16" t="str">
-        <x:v>S</x:v>
+        <x:v>L</x:v>
       </x:c>
       <x:c r="G24" s="14" t="str">
-        <x:v>COM-01</x:v>
+        <x:v>LOAD-01</x:v>
       </x:c>
       <x:c r="H24" s="14" t="str">
         <x:v>Combat Systems</x:v>
       </x:c>
-      <x:c r="I24" s="15" t="str"/>
+      <x:c r="I24" s="15"/>
       <x:c r="J24" s="17" t="str">
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="K24" s="14" t="str">
-        <x:v>The higher roll acts first and a tied result never selects a winner.</x:v>
+        <x:v>A skill is available only when an equipped weapon satisfies every required tag.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="42" customHeight="1">
       <x:c r="A25" s="13" t="str">
-        <x:v>COM-03</x:v>
+        <x:v>INH-01</x:v>
       </x:c>
       <x:c r="B25" s="13" t="str">
-        <x:v>M3 Combat</x:v>
+        <x:v>M2 Party and Loadouts</x:v>
       </x:c>
       <x:c r="C25" s="13" t="str">
-        <x:v>Player Turn</x:v>
+        <x:v>Inherent Skills</x:v>
       </x:c>
       <x:c r="D25" s="14" t="str">
-        <x:v>Implement player movement, skip movement, and action selection.</x:v>
+        <x:v>Implement character-bound passive Inherent Skill definitions and one MVP slot per character.</x:v>
       </x:c>
       <x:c r="E25" s="16" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F25" s="16" t="str">
-        <x:v>L</x:v>
+        <x:v>M</x:v>
       </x:c>
       <x:c r="G25" s="14" t="str">
-        <x:v>COM-01, HEX-04</x:v>
+        <x:v>PARTY-01, DATA-01</x:v>
       </x:c>
       <x:c r="H25" s="14" t="str">
-        <x:v>Combat Systems</x:v>
+        <x:v>Progression</x:v>
       </x:c>
       <x:c r="I25" s="15" t="str"/>
       <x:c r="J25" s="17" t="str">
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="K25" s="14" t="str">
-        <x:v>The player receives one movement phase and one action, and invalid input consumes neither.</x:v>
+        <x:v>An acquired Inherent Skill affects only its owner and cannot enter shared inventory or another character's loadout.</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="42" customHeight="1">
       <x:c r="A26" s="13" t="str">
-        <x:v>COM-04</x:v>
+        <x:v>EVT-01</x:v>
       </x:c>
       <x:c r="B26" s="13" t="str">
-        <x:v>M3 Combat</x:v>
+        <x:v>M2 Party and Loadouts</x:v>
       </x:c>
       <x:c r="C26" s="13" t="str">
-        <x:v>Attack Rules</x:v>
+        <x:v>Event Outcomes</x:v>
       </x:c>
       <x:c r="D26" s="14" t="str">
-        <x:v>Implement attack rolls, Armor Class checks, damage dice, and HP changes.</x:v>
+        <x:v>Implement responder selection and a general event result model for equipment, consumables, resources, Inherent Skills, benefits, and negative consequences.</x:v>
       </x:c>
       <x:c r="E26" s="16" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F26" s="16" t="str">
-        <x:v>M</x:v>
+        <x:v>L</x:v>
       </x:c>
       <x:c r="G26" s="14" t="str">
-        <x:v>COM-01, DATA-01</x:v>
+        <x:v>INH-01, ROOM-05</x:v>
       </x:c>
       <x:c r="H26" s="14" t="str">
-        <x:v>Combat Systems</x:v>
+        <x:v>Progression and UI</x:v>
       </x:c>
       <x:c r="I26" s="15" t="str"/>
       <x:c r="J26" s="17" t="str">
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="K26" s="14" t="str">
-        <x:v>Hit, miss, damage, and zero-HP results match the approved formulas.</x:v>
+        <x:v>An event applies the selected result type; an Inherent Skill reward binds only to the receiving responder.</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="42" customHeight="1">
       <x:c r="A27" s="13" t="str">
-        <x:v>COM-05</x:v>
+        <x:v>INH-02</x:v>
       </x:c>
       <x:c r="B27" s="13" t="str">
-        <x:v>M3 Combat</x:v>
+        <x:v>M2 Party and Loadouts</x:v>
       </x:c>
       <x:c r="C27" s="13" t="str">
-        <x:v>Potion Action</x:v>
+        <x:v>Combat Learning</x:v>
       </x:c>
       <x:c r="D27" s="14" t="str">
-        <x:v>Implement potion use during combat and outside combat.</x:v>
+        <x:v>Record per-character combat behavior and award one eligible post-combat Inherent Skill.</x:v>
       </x:c>
       <x:c r="E27" s="16" t="str">
-        <x:v>P1</x:v>
+        <x:v>P0</x:v>
       </x:c>
       <x:c r="F27" s="16" t="str">
-        <x:v>M</x:v>
+        <x:v>L</x:v>
       </x:c>
       <x:c r="G27" s="14" t="str">
-        <x:v>COM-03, SET-04</x:v>
+        <x:v>INH-01, COM-06</x:v>
       </x:c>
       <x:c r="H27" s="14" t="str">
-        <x:v>Systems</x:v>
+        <x:v>Progression</x:v>
       </x:c>
       <x:c r="I27" s="15" t="str"/>
       <x:c r="J27" s="17" t="str">
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="K27" s="14" t="str">
-        <x:v>A potion heals up to 20 HP, never exceeds maximum HP, and consumes a combat action.</x:v>
+        <x:v>Finishing blows and damage tags are attributed to the correct character and can award the matching Inherent Skill.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="42" customHeight="1">
       <x:c r="A28" s="13" t="str">
-        <x:v>COM-06</x:v>
+        <x:v>COM-01</x:v>
       </x:c>
       <x:c r="B28" s="13" t="str">
         <x:v>M3 Combat</x:v>
       </x:c>
       <x:c r="C28" s="13" t="str">
-        <x:v>Enemy Turn</x:v>
+        <x:v>Encounter Transition</x:v>
       </x:c>
       <x:c r="D28" s="14" t="str">
-        <x:v>Implement enemy range checks, movement, and attack behavior.</x:v>
+        <x:v>Suspend exploration, place the full party and enemies at anchors, and blend to a fixed battle camera.</x:v>
       </x:c>
       <x:c r="E28" s="16" t="str">
         <x:v>P0</x:v>
@@ -1199,64 +1199,64 @@
         <x:v>L</x:v>
       </x:c>
       <x:c r="G28" s="14" t="str">
-        <x:v>COM-01, COM-04, HEX-05</x:v>
+        <x:v>ROOM-02, PARTY-01</x:v>
       </x:c>
       <x:c r="H28" s="14" t="str">
-        <x:v>Combat Systems</x:v>
-      </x:c>
-      <x:c r="I28" s="15" t="str"/>
+        <x:v>Combat and Camera</x:v>
+      </x:c>
+      <x:c r="I28" s="15"/>
       <x:c r="J28" s="17" t="str">
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="K28" s="14" t="str">
-        <x:v>The enemy attacks in range or moves toward the player and attacks when newly in range.</x:v>
+        <x:v>An encounter enters battle without loading another room and every combatant is framed correctly.</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="42" customHeight="1">
       <x:c r="A29" s="13" t="str">
-        <x:v>COM-07</x:v>
+        <x:v>COM-02</x:v>
       </x:c>
       <x:c r="B29" s="13" t="str">
         <x:v>M3 Combat</x:v>
       </x:c>
       <x:c r="C29" s="13" t="str">
-        <x:v>Combat Results</x:v>
+        <x:v>Combat Flow</x:v>
       </x:c>
       <x:c r="D29" s="14" t="str">
-        <x:v>Implement victory, defeat, normal rewards, and boss completion transitions.</x:v>
+        <x:v>Implement CombatController with explicit setup, turn, action, optional interaction, outcome, and exit phases.</x:v>
       </x:c>
       <x:c r="E29" s="16" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F29" s="16" t="str">
-        <x:v>M</x:v>
+        <x:v>L</x:v>
       </x:c>
       <x:c r="G29" s="14" t="str">
-        <x:v>COM-04, COM-06</x:v>
+        <x:v>COM-01</x:v>
       </x:c>
       <x:c r="H29" s="14" t="str">
-        <x:v>Systems</x:v>
+        <x:v>Combat Systems</x:v>
       </x:c>
       <x:c r="I29" s="15" t="str"/>
       <x:c r="J29" s="17" t="str">
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="K29" s="14" t="str">
-        <x:v>Combat ends exactly once and opens the correct result, defeat, or completion state.</x:v>
+        <x:v>One controller owns phase transitions and rejects commands that are invalid for the active phase.</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="42" customHeight="1">
       <x:c r="A30" s="13" t="str">
-        <x:v>COM-08</x:v>
+        <x:v>COM-03</x:v>
       </x:c>
       <x:c r="B30" s="13" t="str">
         <x:v>M3 Combat</x:v>
       </x:c>
       <x:c r="C30" s="13" t="str">
-        <x:v>Retry</x:v>
+        <x:v>Turn Order</x:v>
       </x:c>
       <x:c r="D30" s="14" t="str">
-        <x:v>Capture and restore the complete pre-combat retry snapshot.</x:v>
+        <x:v>Implement deterministic Speed-based turn order with a stable tie-break rule.</x:v>
       </x:c>
       <x:c r="E30" s="16" t="str">
         <x:v>P0</x:v>
@@ -1265,31 +1265,31 @@
         <x:v>M</x:v>
       </x:c>
       <x:c r="G30" s="14" t="str">
-        <x:v>SET-04, COM-07</x:v>
+        <x:v>COM-02, PARTY-02</x:v>
       </x:c>
       <x:c r="H30" s="14" t="str">
-        <x:v>Systems</x:v>
-      </x:c>
-      <x:c r="I30" s="15" t="str"/>
+        <x:v>Combat Systems</x:v>
+      </x:c>
+      <x:c r="I30" s="15"/>
       <x:c r="J30" s="17" t="str">
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="K30" s="14" t="str">
-        <x:v>Retry restores HP, maximum HP, EXP, gold, potions, weapon, and stage state.</x:v>
+        <x:v>The same combat state always produces the same complete turn order.</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="42" customHeight="1">
       <x:c r="A31" s="13" t="str">
-        <x:v>COM-09</x:v>
+        <x:v>COM-04</x:v>
       </x:c>
       <x:c r="B31" s="13" t="str">
         <x:v>M3 Combat</x:v>
       </x:c>
       <x:c r="C31" s="13" t="str">
-        <x:v>Combat UI</x:v>
+        <x:v>Actions and Targets</x:v>
       </x:c>
       <x:c r="D31" s="14" t="str">
-        <x:v>Build the combat HUD, turn indicator, highlights, action controls, and combat log.</x:v>
+        <x:v>Implement one action per turn with skills, item, defend, currently supported optional interaction, and valid target selection.</x:v>
       </x:c>
       <x:c r="E31" s="16" t="str">
         <x:v>P0</x:v>
@@ -1298,460 +1298,460 @@
         <x:v>L</x:v>
       </x:c>
       <x:c r="G31" s="14" t="str">
-        <x:v>COM-03, COM-04, COM-06</x:v>
+        <x:v>COM-02, SKILL-01</x:v>
       </x:c>
       <x:c r="H31" s="14" t="str">
-        <x:v>UI</x:v>
+        <x:v>Combat Systems</x:v>
       </x:c>
       <x:c r="I31" s="15" t="str"/>
       <x:c r="J31" s="17" t="str">
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="K31" s="14" t="str">
-        <x:v>The player can identify the active turn, legal actions, unit stats, and every roll result.</x:v>
+        <x:v>There is no movement command and invalid targets or actions do not consume the turn.</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="42" customHeight="1">
       <x:c r="A32" s="13" t="str">
-        <x:v>NODE-01</x:v>
+        <x:v>COM-05</x:v>
       </x:c>
       <x:c r="B32" s="13" t="str">
-        <x:v>M4 Meta Nodes</x:v>
+        <x:v>M3 Combat</x:v>
       </x:c>
       <x:c r="C32" s="13" t="str">
-        <x:v>Shop</x:v>
+        <x:v>Damage Types</x:v>
       </x:c>
       <x:c r="D32" s="14" t="str">
-        <x:v>Implement potion and weapon purchases with price and purchase limits.</x:v>
+        <x:v>Implement Slashing, Blunt, Piercing, Fire, Ice, Lightning, and data-driven resistance multipliers.</x:v>
       </x:c>
       <x:c r="E32" s="16" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F32" s="16" t="str">
-        <x:v>M</x:v>
+        <x:v>L</x:v>
       </x:c>
       <x:c r="G32" s="14" t="str">
-        <x:v>FLOW-02, DATA-01</x:v>
+        <x:v>COM-04, DATA-01</x:v>
       </x:c>
       <x:c r="H32" s="14" t="str">
-        <x:v>UI and Systems</x:v>
-      </x:c>
-      <x:c r="I32" s="15" t="str"/>
+        <x:v>Combat Systems</x:v>
+      </x:c>
+      <x:c r="I32" s="15"/>
       <x:c r="J32" s="17" t="str">
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="K32" s="14" t="str">
-        <x:v>Purchases enforce gold costs, per-visit limits, and weapon replacement.</x:v>
+        <x:v>All six types resolve through one stable formula and read the correct resistance entry.</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="42" customHeight="1">
       <x:c r="A33" s="13" t="str">
-        <x:v>NODE-02</x:v>
+        <x:v>COM-06</x:v>
       </x:c>
       <x:c r="B33" s="13" t="str">
-        <x:v>M4 Meta Nodes</x:v>
+        <x:v>M3 Combat</x:v>
       </x:c>
       <x:c r="C33" s="13" t="str">
-        <x:v>Reward</x:v>
+        <x:v>Skill Resolution</x:v>
       </x:c>
       <x:c r="D33" s="14" t="str">
-        <x:v>Implement the 50 percent potion or weapon reward node.</x:v>
+        <x:v>Resolve weapon requirements, direct effects, passive modifiers, combat events, optional interactions, and character learning records.</x:v>
       </x:c>
       <x:c r="E33" s="16" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F33" s="16" t="str">
-        <x:v>S</x:v>
+        <x:v>L</x:v>
       </x:c>
       <x:c r="G33" s="14" t="str">
-        <x:v>FLOW-02, DATA-01</x:v>
+        <x:v>COM-04, COM-05</x:v>
       </x:c>
       <x:c r="H33" s="14" t="str">
-        <x:v>Systems</x:v>
+        <x:v>Combat Systems</x:v>
       </x:c>
       <x:c r="I33" s="15" t="str"/>
       <x:c r="J33" s="17" t="str">
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="K33" s="14" t="str">
-        <x:v>The node grants exactly one valid reward and applies weapon replacement correctly.</x:v>
+        <x:v>Resolution produces one ordered result used by HP, presentation, approved extensions, and learning systems.</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="42" customHeight="1">
       <x:c r="A34" s="13" t="str">
-        <x:v>NODE-03</x:v>
+        <x:v>COM-07</x:v>
       </x:c>
       <x:c r="B34" s="13" t="str">
-        <x:v>M4 Meta Nodes</x:v>
+        <x:v>M3 Combat</x:v>
       </x:c>
       <x:c r="C34" s="13" t="str">
-        <x:v>Event</x:v>
+        <x:v>Enemy AI</x:v>
       </x:c>
       <x:c r="D34" s="14" t="str">
-        <x:v>Implement Event 1 choices and Constitution check.</x:v>
+        <x:v>Implement deterministic enemy action scoring for available skills and targets.</x:v>
       </x:c>
       <x:c r="E34" s="16" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F34" s="16" t="str">
-        <x:v>M</x:v>
+        <x:v>L</x:v>
       </x:c>
       <x:c r="G34" s="14" t="str">
-        <x:v>FLOW-02, DATA-02</x:v>
+        <x:v>COM-04, COM-06</x:v>
       </x:c>
       <x:c r="H34" s="14" t="str">
-        <x:v>UI and Systems</x:v>
-      </x:c>
-      <x:c r="I34" s="15" t="str"/>
+        <x:v>Combat Systems</x:v>
+      </x:c>
+      <x:c r="I34" s="15"/>
       <x:c r="J34" s="17" t="str">
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="K34" s="14" t="str">
-        <x:v>All three Event 1 choices apply the approved costs, check, rewards, and damage.</x:v>
+        <x:v>Enemies choose and resolve legal actions without movement or player input.</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="42" customHeight="1">
       <x:c r="A35" s="13" t="str">
-        <x:v>NODE-04</x:v>
+        <x:v>COM-08</x:v>
       </x:c>
       <x:c r="B35" s="13" t="str">
-        <x:v>M4 Meta Nodes</x:v>
+        <x:v>M3 Combat</x:v>
       </x:c>
       <x:c r="C35" s="13" t="str">
-        <x:v>Event</x:v>
+        <x:v>Results and Retry</x:v>
       </x:c>
       <x:c r="D35" s="14" t="str">
-        <x:v>Implement Event 2 choices and Strength check.</x:v>
+        <x:v>Implement victory, defeat, rewards, camera return, and complete pre-combat snapshot restore.</x:v>
       </x:c>
       <x:c r="E35" s="16" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F35" s="16" t="str">
-        <x:v>M</x:v>
+        <x:v>L</x:v>
       </x:c>
       <x:c r="G35" s="14" t="str">
-        <x:v>FLOW-02, DATA-02</x:v>
+        <x:v>COM-06, COM-07, SET-04</x:v>
       </x:c>
       <x:c r="H35" s="14" t="str">
-        <x:v>UI and Systems</x:v>
+        <x:v>Systems</x:v>
       </x:c>
       <x:c r="I35" s="15" t="str"/>
       <x:c r="J35" s="17" t="str">
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="K35" s="14" t="str">
-        <x:v>All three Event 2 choices apply the approved weapon, HP, maximum HP, and gold results.</x:v>
+        <x:v>Retry restores party, loadout, Inherent Skills, room interactions, event rewards, encounter state, and approved optional state.</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="42" customHeight="1">
       <x:c r="A36" s="13" t="str">
-        <x:v>PROG-01</x:v>
+        <x:v>COM-09</x:v>
       </x:c>
       <x:c r="B36" s="13" t="str">
-        <x:v>M4 Meta Nodes</x:v>
+        <x:v>M3 Combat</x:v>
       </x:c>
       <x:c r="C36" s="13" t="str">
-        <x:v>Progression</x:v>
+        <x:v>Combat UI</x:v>
       </x:c>
       <x:c r="D36" s="14" t="str">
-        <x:v>Implement EXP gain and leveling without healing current HP.</x:v>
+        <x:v>Build party and enemy status, turn order, action selection, targeting, previews, and combat log.</x:v>
       </x:c>
       <x:c r="E36" s="16" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F36" s="16" t="str">
-        <x:v>S</x:v>
+        <x:v>L</x:v>
       </x:c>
       <x:c r="G36" s="14" t="str">
-        <x:v>SET-04, COM-07</x:v>
+        <x:v>COM-04, COM-06</x:v>
       </x:c>
       <x:c r="H36" s="14" t="str">
-        <x:v>Systems</x:v>
-      </x:c>
-      <x:c r="I36" s="15" t="str"/>
+        <x:v>UI</x:v>
+      </x:c>
+      <x:c r="I36" s="15"/>
       <x:c r="J36" s="17" t="str">
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="K36" s="14" t="str">
-        <x:v>Every 10 EXP increases maximum HP by 5 and preserves current HP.</x:v>
+        <x:v>The player can identify the active actor, legal actions, targets, costs, types, and resolved effects.</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="42" customHeight="1">
       <x:c r="A37" s="13" t="str">
-        <x:v>PROG-02</x:v>
+        <x:v>ENV-01</x:v>
       </x:c>
       <x:c r="B37" s="13" t="str">
-        <x:v>M4 Meta Nodes</x:v>
+        <x:v>M4 Environment and Activities</x:v>
       </x:c>
       <x:c r="C37" s="13" t="str">
-        <x:v>Weapons</x:v>
+        <x:v>Environment Extension</x:v>
       </x:c>
       <x:c r="D37" s="14" t="str">
-        <x:v>Implement accuracy and damage weapon effects with replacement behavior.</x:v>
+        <x:v>Add a small optional data-driven hook for environment interactions without defining a complete environment system.</x:v>
       </x:c>
       <x:c r="E37" s="16" t="str">
-        <x:v>P0</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="F37" s="16" t="str">
         <x:v>M</x:v>
       </x:c>
       <x:c r="G37" s="14" t="str">
-        <x:v>DATA-01, COM-04</x:v>
+        <x:v>COM-02, DATA-01</x:v>
       </x:c>
       <x:c r="H37" s="14" t="str">
-        <x:v>Systems</x:v>
+        <x:v>Environment Systems</x:v>
       </x:c>
       <x:c r="I37" s="15" t="str"/>
       <x:c r="J37" s="17" t="str">
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="K37" s="14" t="str">
-        <x:v>Accuracy produces a total +4 attack bonus and damage changes from 1D10 to 2D10.</x:v>
+        <x:v>Core combat works unchanged when no environment interaction definition is assigned.</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="42" customHeight="1">
       <x:c r="A38" s="13" t="str">
-        <x:v>PROG-03</x:v>
+        <x:v>ENV-02</x:v>
       </x:c>
       <x:c r="B38" s="13" t="str">
-        <x:v>M4 Meta Nodes</x:v>
+        <x:v>M4 Environment and Activities</x:v>
       </x:c>
       <x:c r="C38" s="13" t="str">
-        <x:v>Rewards</x:v>
+        <x:v>Provisional Examples</x:v>
       </x:c>
       <x:c r="D38" s="14" t="str">
-        <x:v>Implement 5 gold, 5 EXP, and 25 percent potion combat rewards.</x:v>
+        <x:v>Create editable placeholder definitions for Oil + Fire and Water + Lightning and label both as provisional.</x:v>
       </x:c>
       <x:c r="E38" s="16" t="str">
-        <x:v>P0</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="F38" s="16" t="str">
         <x:v>S</x:v>
       </x:c>
       <x:c r="G38" s="14" t="str">
-        <x:v>COM-07, PROG-01</x:v>
+        <x:v>ENV-01</x:v>
       </x:c>
       <x:c r="H38" s="14" t="str">
-        <x:v>Systems</x:v>
+        <x:v>Design and Systems</x:v>
       </x:c>
       <x:c r="I38" s="15" t="str"/>
       <x:c r="J38" s="17" t="str">
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="K38" s="14" t="str">
-        <x:v>Normal victory applies each reward exactly once and displays the actual result.</x:v>
+        <x:v>Both examples can be reviewed without establishing final effects, targeting rules, or MVP inclusion.</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="42" customHeight="1">
       <x:c r="A39" s="13" t="str">
-        <x:v>BOSS-01</x:v>
+        <x:v>ENV-03</x:v>
       </x:c>
       <x:c r="B39" s="13" t="str">
-        <x:v>M5 Integration and QA</x:v>
+        <x:v>M4 Environment and Activities</x:v>
       </x:c>
       <x:c r="C39" s="13" t="str">
-        <x:v>Boss</x:v>
+        <x:v>Team Decision</x:v>
       </x:c>
       <x:c r="D39" s="14" t="str">
-        <x:v>Configure Stage 1-5 boss statistics and boss-specific completion behavior.</x:v>
+        <x:v>Review the provisional examples and record whether each is approved, revised, replaced, or removed.</x:v>
       </x:c>
       <x:c r="E39" s="16" t="str">
-        <x:v>P0</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="F39" s="16" t="str">
         <x:v>S</x:v>
       </x:c>
       <x:c r="G39" s="14" t="str">
-        <x:v>COM-07, DATA-02</x:v>
+        <x:v>ENV-02</x:v>
       </x:c>
       <x:c r="H39" s="14" t="str">
-        <x:v>Combat Systems</x:v>
+        <x:v>Whole Team</x:v>
       </x:c>
       <x:c r="I39" s="15" t="str"/>
       <x:c r="J39" s="17" t="str">
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="K39" s="14" t="str">
-        <x:v>The boss uses 80 HP, AC 7, +2 attack, 2D4 damage, and opens RunComplete on victory.</x:v>
+        <x:v>The backlog and specification reflect the team's decision before implementation begins.</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="42" customHeight="1">
       <x:c r="A40" s="13" t="str">
-        <x:v>UI-01</x:v>
+        <x:v>ENV-04</x:v>
       </x:c>
       <x:c r="B40" s="13" t="str">
-        <x:v>M5 Integration and QA</x:v>
+        <x:v>M4 Environment and Activities</x:v>
       </x:c>
       <x:c r="C40" s="13" t="str">
-        <x:v>Menu UI</x:v>
+        <x:v>Oil and Fire Prototype</x:v>
       </x:c>
       <x:c r="D40" s="14" t="str">
-        <x:v>Build the main menu and Start Game action.</x:v>
+        <x:v>If approved, implement the team-defined Oil + Fire behavior through the optional interaction hook.</x:v>
       </x:c>
       <x:c r="E40" s="16" t="str">
-        <x:v>P0</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="F40" s="16" t="str">
-        <x:v>S</x:v>
+        <x:v>M</x:v>
       </x:c>
       <x:c r="G40" s="14" t="str">
-        <x:v>SET-03, FLOW-03</x:v>
+        <x:v>ENV-03, COM-05</x:v>
       </x:c>
       <x:c r="H40" s="14" t="str">
-        <x:v>UI</x:v>
+        <x:v>Environment Systems</x:v>
       </x:c>
       <x:c r="I40" s="15" t="str"/>
       <x:c r="J40" s="17" t="str">
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="K40" s="14" t="str">
-        <x:v>Start Game initializes a clean run and opens Stage 1-1.</x:v>
+        <x:v>The prototype matches the approved definition and adds no unapproved environment rules.</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="42" customHeight="1">
       <x:c r="A41" s="13" t="str">
-        <x:v>UI-02</x:v>
+        <x:v>ENV-05</x:v>
       </x:c>
       <x:c r="B41" s="13" t="str">
-        <x:v>M5 Integration and QA</x:v>
+        <x:v>M4 Environment and Activities</x:v>
       </x:c>
       <x:c r="C41" s="13" t="str">
-        <x:v>Result UI</x:v>
+        <x:v>Water and Lightning Prototype</x:v>
       </x:c>
       <x:c r="D41" s="14" t="str">
-        <x:v>Build normal result, defeat, and retry panels.</x:v>
+        <x:v>If approved, implement the team-defined Water + Lightning behavior through the optional interaction hook.</x:v>
       </x:c>
       <x:c r="E41" s="16" t="str">
-        <x:v>P0</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="F41" s="16" t="str">
         <x:v>M</x:v>
       </x:c>
       <x:c r="G41" s="14" t="str">
-        <x:v>COM-07, COM-08</x:v>
+        <x:v>ENV-03, COM-05</x:v>
       </x:c>
       <x:c r="H41" s="14" t="str">
-        <x:v>UI</x:v>
+        <x:v>Environment Systems</x:v>
       </x:c>
       <x:c r="I41" s="15" t="str"/>
       <x:c r="J41" s="17" t="str">
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="K41" s="14" t="str">
-        <x:v>Each panel shows the correct information and exposes only valid actions.</x:v>
+        <x:v>The prototype matches the approved definition and adds no unapproved environment rules.</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="42" customHeight="1">
       <x:c r="A42" s="13" t="str">
-        <x:v>UI-03</x:v>
+        <x:v>ENV-06</x:v>
       </x:c>
       <x:c r="B42" s="13" t="str">
-        <x:v>M5 Integration and QA</x:v>
+        <x:v>M4 Environment and Activities</x:v>
       </x:c>
       <x:c r="C42" s="13" t="str">
-        <x:v>Completion UI</x:v>
+        <x:v>Environment Feedback</x:v>
       </x:c>
       <x:c r="D42" s="14" t="str">
-        <x:v>Build the run-complete screen and return-to-menu action.</x:v>
+        <x:v>If an example is retained, show only the feedback needed to understand its approved effect.</x:v>
       </x:c>
       <x:c r="E42" s="16" t="str">
-        <x:v>P0</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="F42" s="16" t="str">
-        <x:v>S</x:v>
+        <x:v>M</x:v>
       </x:c>
       <x:c r="G42" s="14" t="str">
-        <x:v>BOSS-01, FLOW-03</x:v>
+        <x:v>ENV-04, ENV-05, COM-09</x:v>
       </x:c>
       <x:c r="H42" s="14" t="str">
-        <x:v>UI</x:v>
+        <x:v>UI and VFX</x:v>
       </x:c>
       <x:c r="I42" s="15" t="str"/>
       <x:c r="J42" s="17" t="str">
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="K42" s="14" t="str">
-        <x:v>Boss victory opens the screen and returning to the menu clears the run.</x:v>
+        <x:v>Retained interactions are readable without implying a broader finalized environment system.</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="42" customHeight="1">
       <x:c r="A43" s="13" t="str">
-        <x:v>QA-01</x:v>
+        <x:v>ACT-01</x:v>
       </x:c>
       <x:c r="B43" s="13" t="str">
-        <x:v>M5 Integration and QA</x:v>
+        <x:v>M4 Environment and Activities</x:v>
       </x:c>
       <x:c r="C43" s="13" t="str">
-        <x:v>EditMode Tests</x:v>
+        <x:v>Room Activities</x:v>
       </x:c>
       <x:c r="D43" s="14" t="str">
-        <x:v>Add tests for hex generation, neighbors, distance, movement range, and pathfinding.</x:v>
+        <x:v>Implement one merchant, one chest, and one responder-based event with multiple possible result categories.</x:v>
       </x:c>
       <x:c r="E43" s="16" t="str">
-        <x:v>P1</x:v>
+        <x:v>P0</x:v>
       </x:c>
       <x:c r="F43" s="16" t="str">
-        <x:v>M</x:v>
+        <x:v>L</x:v>
       </x:c>
       <x:c r="G43" s="14" t="str">
-        <x:v>HEX-05</x:v>
+        <x:v>ROOM-05, EVT-01, COM-08</x:v>
       </x:c>
       <x:c r="H43" s="14" t="str">
-        <x:v>QA</x:v>
+        <x:v>UI and Systems</x:v>
       </x:c>
       <x:c r="I43" s="15" t="str"/>
       <x:c r="J43" s="17" t="str">
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="K43" s="14" t="str">
-        <x:v>The grid test suite covers the 37-cell board and representative edge cases.</x:v>
+        <x:v>Activities coexist with encounters, persist results, and events may award equipment, consumables, resources, or an Inherent Skill.</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="42" customHeight="1">
       <x:c r="A44" s="13" t="str">
-        <x:v>QA-02</x:v>
+        <x:v>BOSS-01</x:v>
       </x:c>
       <x:c r="B44" s="13" t="str">
         <x:v>M5 Integration and QA</x:v>
       </x:c>
       <x:c r="C44" s="13" t="str">
-        <x:v>EditMode Tests</x:v>
+        <x:v>Boss and Completion</x:v>
       </x:c>
       <x:c r="D44" s="14" t="str">
-        <x:v>Add tests for stage rules, dice rules, rewards, leveling, events, and retry snapshots.</x:v>
+        <x:v>Configure the boss encounter, final door rules, run-complete screen, and return-to-menu reset.</x:v>
       </x:c>
       <x:c r="E44" s="16" t="str">
-        <x:v>P1</x:v>
+        <x:v>P0</x:v>
       </x:c>
       <x:c r="F44" s="16" t="str">
-        <x:v>L</x:v>
+        <x:v>M</x:v>
       </x:c>
       <x:c r="G44" s="14" t="str">
-        <x:v>FLOW-01, COM-08, NODE-04, PROG-03</x:v>
+        <x:v>ROOM-07, COM-08</x:v>
       </x:c>
       <x:c r="H44" s="14" t="str">
-        <x:v>QA</x:v>
+        <x:v>Combat and UI</x:v>
       </x:c>
       <x:c r="I44" s="15" t="str"/>
       <x:c r="J44" s="17" t="str">
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="K44" s="14" t="str">
-        <x:v>Tests cover every approved rule and fail when a boundary condition is intentionally broken.</x:v>
+        <x:v>Boss victory ends the run once and returning to menu clears every runtime state.</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="42" customHeight="1">
       <x:c r="A45" s="13" t="str">
-        <x:v>QA-03</x:v>
+        <x:v>QA-01</x:v>
       </x:c>
       <x:c r="B45" s="13" t="str">
         <x:v>M5 Integration and QA</x:v>
       </x:c>
       <x:c r="C45" s="13" t="str">
-        <x:v>PlayMode Tests</x:v>
+        <x:v>EditMode Tests</x:v>
       </x:c>
       <x:c r="D45" s="14" t="str">
-        <x:v>Add smoke tests for new run, combat return, boss completion, and run reset.</x:v>
+        <x:v>Add tests for rooms, doors, turn order, skill requirements, damage types, event result categories, Inherent Skills, and retry.</x:v>
       </x:c>
       <x:c r="E45" s="16" t="str">
         <x:v>P1</x:v>
@@ -1760,7 +1760,7 @@
         <x:v>L</x:v>
       </x:c>
       <x:c r="G45" s="14" t="str">
-        <x:v>UI-03, QA-02</x:v>
+        <x:v>INH-02, COM-08, EVT-01</x:v>
       </x:c>
       <x:c r="H45" s="14" t="str">
         <x:v>QA</x:v>
@@ -1770,40 +1770,40 @@
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="K45" s="14" t="str">
-        <x:v>The critical scene flow completes without exceptions in PlayMode tests.</x:v>
+        <x:v>Tests cover deterministic rules, reward types, character ownership, retry state, and representative boundary cases.</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="42" customHeight="1">
       <x:c r="A46" s="13" t="str">
-        <x:v>QA-04</x:v>
+        <x:v>QA-02</x:v>
       </x:c>
       <x:c r="B46" s="13" t="str">
         <x:v>M5 Integration and QA</x:v>
       </x:c>
       <x:c r="C46" s="13" t="str">
-        <x:v>Acceptance Test</x:v>
+        <x:v>PlayMode Tests</x:v>
       </x:c>
       <x:c r="D46" s="14" t="str">
-        <x:v>Run the complete MVP acceptance checklist and record defects.</x:v>
+        <x:v>Add smoke tests for new run, door transition, camera transition, mixed activities, retry, boss completion, and reset.</x:v>
       </x:c>
       <x:c r="E46" s="16" t="str">
-        <x:v>P0</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="F46" s="16" t="str">
         <x:v>L</x:v>
       </x:c>
       <x:c r="G46" s="14" t="str">
-        <x:v>QA-01, QA-03</x:v>
+        <x:v>ACT-01, BOSS-01, QA-01</x:v>
       </x:c>
       <x:c r="H46" s="14" t="str">
-        <x:v>Whole Team</x:v>
-      </x:c>
-      <x:c r="I46" s="15" t="str"/>
+        <x:v>QA</x:v>
+      </x:c>
+      <x:c r="I46" s="15"/>
       <x:c r="J46" s="17" t="str">
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="K46" s="14" t="str">
-        <x:v>All specification acceptance criteria pass or have documented blocking defects.</x:v>
+        <x:v>The critical three-room flow completes without exceptions and restores the correct state after retry.</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="42" customHeight="1">
@@ -1814,29 +1814,29 @@
         <x:v>M5 Integration and QA</x:v>
       </x:c>
       <x:c r="C47" s="13" t="str">
-        <x:v>Documentation</x:v>
+        <x:v>Acceptance and Documentation</x:v>
       </x:c>
       <x:c r="D47" s="14" t="str">
-        <x:v>Update team documents and diagrams after implementation decisions change.</x:v>
+        <x:v>Run the v2.0 acceptance checklist and keep the specification, diagrams, and backlog aligned with the delivered slice.</x:v>
       </x:c>
       <x:c r="E47" s="16" t="str">
-        <x:v>P1</x:v>
+        <x:v>P0</x:v>
       </x:c>
       <x:c r="F47" s="16" t="str">
-        <x:v>S</x:v>
+        <x:v>L</x:v>
       </x:c>
       <x:c r="G47" s="14" t="str">
-        <x:v>QA-04</x:v>
+        <x:v>QA-02</x:v>
       </x:c>
       <x:c r="H47" s="14" t="str">
-        <x:v>Tech Lead</x:v>
-      </x:c>
-      <x:c r="I47" s="15" t="str"/>
+        <x:v>Whole Team</x:v>
+      </x:c>
+      <x:c r="I47" s="15"/>
       <x:c r="J47" s="17" t="str">
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="K47" s="14" t="str">
-        <x:v>The specification, architecture, diagrams, and backlog match the delivered build.</x:v>
+        <x:v>Every acceptance criterion passes or has a documented blocking defect and all team documents match the build.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1863,7 +1863,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c8916301c784470"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rffacdba7defa402c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>